<commit_message>
feat: recuperacao retroativa de 34 datas (24/08 a 26/09) resgatando 193 lojas e 11448 pedidos (19602 e 19693 regularizadas)
</commit_message>
<xml_diff>
--- a/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-08-24).xlsx
+++ b/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-08-24).xlsx
@@ -935,13 +935,13 @@
     <t>214</t>
   </si>
   <si>
-    <t>19</t>
+    <t>17</t>
   </si>
   <si>
-    <t>R$ 2.993,83</t>
+    <t>R$ 2.977,15</t>
   </si>
   <si>
-    <t>33.9</t>
+    <t>33.7</t>
   </si>
   <si>
     <t>21.5</t>
@@ -950,16 +950,16 @@
     <t>4.70</t>
   </si>
   <si>
-    <t>17.8</t>
+    <t>18.1</t>
   </si>
   <si>
-    <t>6.3</t>
+    <t>6.6</t>
   </si>
   <si>
     <t>6.4</t>
   </si>
   <si>
-    <t>46.5%</t>
+    <t>46.6%</t>
   </si>
   <si>
     <t>18.5%</t>
@@ -6855,7 +6855,7 @@
         <v>19562</v>
       </c>
       <c r="B36" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C36" s="4">
         <v>51</v>
@@ -6885,14 +6885,26 @@
         <v>58</v>
       </c>
       <c r="L36" s="4"/>
-      <c r="M36" s="5"/>
-      <c r="N36" s="6"/>
+      <c r="M36" s="5">
+        <v>2178</v>
+      </c>
+      <c r="N36" s="6">
+        <v>29</v>
+      </c>
       <c r="O36" s="6"/>
-      <c r="P36" s="7"/>
-      <c r="Q36" s="8"/>
-      <c r="R36" s="8"/>
+      <c r="P36" s="7">
+        <v>6.5488107142857146</v>
+      </c>
+      <c r="Q36" s="8">
+        <v>18.469605882352941</v>
+      </c>
+      <c r="R36" s="8">
+        <v>8.5212090909090907</v>
+      </c>
       <c r="S36" s="8"/>
-      <c r="T36" s="9"/>
+      <c r="T36" s="9">
+        <v>0.29411764705882354</v>
+      </c>
       <c r="U36" s="9"/>
       <c r="V36" s="9"/>
       <c r="W36" s="9"/>
@@ -9144,7 +9156,7 @@
         <v>19602</v>
       </c>
       <c r="B51" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C51" s="4">
         <v>51</v>
@@ -9174,14 +9186,26 @@
         <v>58</v>
       </c>
       <c r="L51" s="4"/>
-      <c r="M51" s="5"/>
-      <c r="N51" s="6"/>
+      <c r="M51" s="5">
+        <v>523.44000000000005</v>
+      </c>
+      <c r="N51" s="6">
+        <v>5</v>
+      </c>
       <c r="O51" s="6"/>
-      <c r="P51" s="7"/>
-      <c r="Q51" s="8"/>
-      <c r="R51" s="8"/>
+      <c r="P51" s="7">
+        <v>2.61334</v>
+      </c>
+      <c r="Q51" s="8">
+        <v>66.400000000000006</v>
+      </c>
+      <c r="R51" s="8">
+        <v>57.375</v>
+      </c>
       <c r="S51" s="8"/>
-      <c r="T51" s="9"/>
+      <c r="T51" s="9">
+        <v>0</v>
+      </c>
       <c r="U51" s="9"/>
       <c r="V51" s="9"/>
       <c r="W51" s="9"/>

</xml_diff>